<commit_message>
version 2 with all working model
</commit_message>
<xml_diff>
--- a/new_excel.xlsx
+++ b/new_excel.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,11 @@
           <t>Summary Status</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>AI Summary</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -504,7 +509,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>NOT_SUMMARIZED</t>
+          <t>SUMMARIZED</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>The Shiromani Akal Dal’s revival is facing challenges as evidenced by the significant exodus of leaders, particularly in the Doaba region. Protests recently held yielded a small number of recognizable faces, indicating a decline in the party’s popularity. This suggests a serious struggle for the Akal Dal to regain its former influence.</t>
         </is>
       </c>
     </row>
@@ -542,7 +552,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NOT_SUMMARIZED</t>
+          <t>SUMMARIZED</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Mrunal Thakur revealed that “Son of Sardaar 2” marked her first foray into commercial entertainment, thanks to encouragement from Ajay Devgn. The film, a sequel to the 2012 hit, features Thakur playing a comedic role alongside Devgn and a large ensemble cast, including those who fondly remember co-star Mukul Dev. Thakur expressed gratitude for the opportunity and the enjoyable experience of filmin...</t>
         </is>
       </c>
     </row>
@@ -580,7 +595,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NOT_SUMMARIZED</t>
+          <t>SUMMARIZED</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Dyal Singh Majithia hailed from a prominent Sikh family deeply involved in the service of Maharaja Ranjit Singh, with his relatives holding key positions within the kingdom. Leveraging his family’s influence and business acumen, he transitioned from a privileged background to become a successful real estate developer, acquiring and managing properties in Lahore. His career culminated in ownership ...</t>
         </is>
       </c>
     </row>
@@ -618,7 +638,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NOT_SUMMARIZED</t>
+          <t>SUMMARIZED</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>The International Olympic Committee has announced that T20 cricket competitions for men and women will take place at the Pomona Fairplex in Los Angeles from July 12 to July 29, 2028, with medal matches on July 20 and 29.  This marks cricket’s second Olympic appearance after a 128-year hiatus, and will involve 6 teams per category.  Details regarding qualification for the LA28 games are still being...</t>
         </is>
       </c>
     </row>
@@ -656,7 +681,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NOT_SUMMARIZED</t>
+          <t>SUMMARIZED</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>The Artist Event Cricket League (AECL) is launching its 7th season on September 13, 2025, featuring a celebrity team versus Team Samarthanam, the visually challenged cricket champions. The launch event included prominent figures from entertainment, sports, and government, alongside the unveiling of a commemorative book celebrating the league’s history. This season promises a significant cash prize...</t>
         </is>
       </c>
     </row>
@@ -694,7 +724,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NOT_SUMMARIZED</t>
+          <t>SUMMARIZED</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Indian stock indices Sensex and Nifty closed slightly higher due to cautious investor sentiment amid global market weakness and tariff concerns. Tech Mahindra and Infosys were key gainers, particularly with Tech Mahindra’s strong financial results announced after market close. The day’s trading was characterized by a mixed performance, with several large companies experiencing declines.</t>
         </is>
       </c>
     </row>
@@ -732,7 +767,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NOT_SUMMARIZED</t>
+          <t>SUMMARIZED</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>The FBI has identified three senior Iranian intelligence officers – Reza Amiri Moghadam, Taghi Daneshvar, and Gholamhossein Mohammadnia – as playing key roles in the 2007 abduction of Robert Levinson. These individuals, including a former ambassador to Pakistan and Albania, allegedly facilitated Levinson’s disappearance and concealed Iran’s involvement. The FBI continues to pursue accountability f...</t>
         </is>
       </c>
     </row>
@@ -770,7 +810,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NOT_SUMMARIZED</t>
+          <t>SUMMARIZED</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Taiwan’s financial exposure to China decreased significantly by the end of May, dropping nearly 20% to NT$828.39 billion due to concerns about China’s economic slowdown and property market instability. This decline, particularly in interbank loans and investments in marketable securities, resulted in a record low exposure-to-net-worth ratio for Taiwanese banks and insurers. The reduction reflects ...</t>
         </is>
       </c>
     </row>
@@ -808,7 +853,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NOT_SUMMARIZED</t>
+          <t>SUMMARIZED</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>The Union Cabinet approved the Prime Minister Dhan-Dhaanya Krishi Yojana, a program designed to boost agricultural productivity and sustainability across 100 identified districts.  This initiative, costing Rs 24,000 crore annually for six years, will utilize a coordinated approach involving existing schemes and private sector partnerships. The scheme aims to support 1.7 crore farmers through impro...</t>
         </is>
       </c>
     </row>
@@ -846,7 +896,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NOT_SUMMARIZED</t>
+          <t>SUMMARIZED</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>“Chhoriyan Chali Gaon” is a new reality series featuring twelve urban women who will live for 60 days in a traditional Indian village, foregoing modern conveniences and embracing rural life. The show aims to explore cultural immersion, personal transformation, and social dynamics through challenging daily tasks and integration with village customs. Actor Rannvijay Singha will host, emphasizing the...</t>
         </is>
       </c>
     </row>
@@ -887,6 +942,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -925,6 +981,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -963,6 +1020,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1001,6 +1059,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1039,6 +1098,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1077,6 +1137,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1115,6 +1176,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1139,7 +1201,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>The security forces on Wednesday achieved a major success in their operation against Maoists as 27 Naxals, including topmost leader Nambala Keshav Rao, aka Basavaraju, were killed in an encounter in the Abujhmad region of Chhattisgarh on the border of Narayanpur and Bijapur districts. A jawan of the Chhattisgarh Police’s District Reserve Guard (DRG) was also killed while a few other personnel sustained injuries in the encounter that had begun several days ago, sources in the state police said. The killing of Keshav Rao, a CPI-Maoist general secretary, has come as a shot in the arm for the security forces as they had recently busted a long-time base of the Naxalites located in Koreguttalu Hills of Bijapur district in Chhattisgarh (bordering Telangana). Thirtyone Naxals were killed and a huge cache of arms, ammunitions and explosives recovered. Four factories where weapons were being manufactured were also unearthed under the three-week-long offensive named Operation Black Forest. Keshav Raocarried a bounty of Rs 1.5 crore and was wanted in connection with several deadly attacks on security forces across multiple states. A native of Jiyyannapet village in Andhra Pradesh's Srikakulam district, he was the son of a school teacher. He studied engineering at Warangal Regional Engineering College (REC) before being drawn into student activism in the 1980s. After being arrested during a student union protest in 1980, he went underground and joined the Naxals. Over the next four decades, Rao rose through the ranks and became known for his meticulous planning, ruthless ambushes, expertise in jungle warfare and making IEDs. Security officials believe he was the mastermind behind the 2010 Dantewada attack, one of the deadliest ever on Indian forces, in which 76 CRPF jawans were killed in Chhattisgarh. Despite the massive bounty, Rao managed to remain elusive for decades. The National Investigation Agency (NIA) had no recent photographs or confirmed details about his age. Prime M</t>
+          <t>The security forces on Wednesday achieved a major success in their operation against Maoists as 27 Naxals, including topmost leader Nambala Keshav Rao, aka Basavaraju, were killed in an encounter in the Abujhmad region of Chhattisgarh on the border of Narayanpur and Bijapur districts.AdvertisementA jawan of the Chhattisgarh Police’s District Reserve Guard (DRG) was also killed while a few other personnel sustained injuries in the encounter that had begun several days ago, sources in the state police said.The killing of Keshav Rao, a CPI-Maoist general secretary, has come as a shot in the arm for the security forces as they had recently busted a long-time base of the Naxalites located in Koreguttalu Hills of Bijapur district in Chhattisgarh (bordering Telangana). Thirtyone Naxals were killed and a huge cache of arms, ammunitions and explosives recovered. Four factories where weapons were being manufactured were also unearthed under the three-week-long offensive named Operation Black Forest.AdvertisementKeshav Raocarried a bounty of Rs 1.5 crore and was wanted in connection with several deadly attacks on security forces across multiple states. A native of Jiyyannapet village in Andhra Pradesh's Srikakulam district, he was the son of a school teacher. He studied engineering at Warangal Regional Engineering College (REC) before being drawn into student activism in the 1980s.After being arrested during a student union protest in 1980, he went underground and joined the Naxals. Over the next four decades, Rao rose through the ranks and became known for his meticulous planning, ruthless ambushes, expertise in jungle warfare and making IEDs.AdvertisementSecurity officials believe he was the mastermind behind the 2010 Dantewada attack, one of the deadliest ever on Indian forces, in which 76 CRPF jawans were killed in Chhattisgarh. Despite the massive bounty, Rao managed to remain elusive for decades. The National Investigation Agency (NIA) had no recent photographs or confirmed details about his age.Prime Minister Narendra Modi and Home Minister Amit Shah lauded the efforts of the security forces. “A landmark achievement in the battle to eliminate Naxalism. Our security forces have neutralised 27 dreaded Maoists, including Nambala Keshav Rao, alias Basavaraju, the general secretary of CPI-Maoist, topmost leader, and the backbone of the Naxal movement. This is the first time in three decades of Bharat's battle against Naxalism that a general secretary-ranked leader has been neutralised. I applaud our brave security forces for this major breakthrough," Shah said in a post on X.Shah said after the completion of Operation Black Forest, 54 Naxalites had been arrested while 84 had surrendered in Chhattisgarh, Telangana and Maharashtra.Tagging Shah's post, PM Modi said, "Proud of our forces for this remarkable success. Our government is committed to eliminating the menace of Maoism and ensuring a life of peace and progress for our people."×Unlock Exclusive Insig...</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -1153,6 +1215,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1191,6 +1254,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1229,6 +1293,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1267,6 +1332,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1305,6 +1371,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1343,6 +1410,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1381,6 +1449,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1419,6 +1488,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1457,6 +1527,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1495,6 +1566,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1533,6 +1605,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1571,6 +1644,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1609,6 +1683,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1647,6 +1722,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1685,6 +1761,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1723,6 +1800,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1761,6 +1839,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1799,6 +1878,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1837,6 +1917,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1875,6 +1956,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1913,6 +1995,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1951,6 +2034,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1989,6 +2073,7 @@
           <t>NOT_SUMMARIZED</t>
         </is>
       </c>
+      <c r="I41" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>